<commit_message>
Changed RF to MICE for imputation and tweaked the parameters for final Imputation
</commit_message>
<xml_diff>
--- a/DiabetesCleaned.xlsx
+++ b/DiabetesCleaned.xlsx
@@ -610,7 +610,7 @@
         <v>20</v>
       </c>
       <c r="E6" t="n">
-        <v>33.3733621621875</v>
+        <v>37.10472324339428</v>
       </c>
       <c r="F6" t="n">
         <v>24.4</v>
@@ -1909,7 +1909,7 @@
         <v>183</v>
       </c>
       <c r="C51" t="n">
-        <v>77.12114511951675</v>
+        <v>74.60475373802224</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
@@ -2167,7 +2167,7 @@
         <v>1</v>
       </c>
       <c r="B60" t="n">
-        <v>90.62035702479233</v>
+        <v>104.7970651670725</v>
       </c>
       <c r="C60" t="n">
         <v>74</v>
@@ -2199,7 +2199,7 @@
         <v>146</v>
       </c>
       <c r="C61" t="n">
-        <v>76.85950750067865</v>
+        <v>71.57072436881829</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>31.72671117694619</v>
+        <v>30.81547598881929</v>
       </c>
       <c r="G61" t="n">
         <v>0.24</v>
@@ -3214,7 +3214,7 @@
         <v>129</v>
       </c>
       <c r="C96" t="n">
-        <v>111.2695288957292</v>
+        <v>84.52043378662961</v>
       </c>
       <c r="D96" t="n">
         <v>30</v>
@@ -3794,7 +3794,7 @@
         <v>120</v>
       </c>
       <c r="C116" t="n">
-        <v>76.16191024666732</v>
+        <v>75.92283155244778</v>
       </c>
       <c r="D116" t="n">
         <v>0</v>
@@ -5012,7 +5012,7 @@
         <v>114</v>
       </c>
       <c r="C158" t="n">
-        <v>70.43781126521566</v>
+        <v>71.27348197058369</v>
       </c>
       <c r="D158" t="n">
         <v>0</v>
@@ -5021,7 +5021,7 @@
         <v>0</v>
       </c>
       <c r="F158" t="n">
-        <v>29.90296691495914</v>
+        <v>29.31107299630873</v>
       </c>
       <c r="G158" t="n">
         <v>0.189</v>
@@ -5215,7 +5215,7 @@
         <v>141</v>
       </c>
       <c r="C165" t="n">
-        <v>73.74194556935319</v>
+        <v>71.2382792195591</v>
       </c>
       <c r="D165" t="n">
         <v>0</v>
@@ -5592,7 +5592,7 @@
         <v>80</v>
       </c>
       <c r="C178" t="n">
-        <v>66.45442322712771</v>
+        <v>67.55322038110384</v>
       </c>
       <c r="D178" t="n">
         <v>0</v>
@@ -5601,7 +5601,7 @@
         <v>0</v>
       </c>
       <c r="F178" t="n">
-        <v>29.35369501897569</v>
+        <v>27.5349765300166</v>
       </c>
       <c r="G178" t="n">
         <v>0.174</v>
@@ -5969,7 +5969,7 @@
         <v>100</v>
       </c>
       <c r="C191" t="n">
-        <v>70.70684698280897</v>
+        <v>73.33872677059739</v>
       </c>
       <c r="D191" t="n">
         <v>0</v>
@@ -6198,7 +6198,7 @@
         <v>1</v>
       </c>
       <c r="B199" t="n">
-        <v>104.4851832149699</v>
+        <v>101.9041563643626</v>
       </c>
       <c r="C199" t="n">
         <v>68</v>
@@ -6549,7 +6549,7 @@
         <v>180</v>
       </c>
       <c r="C211" t="n">
-        <v>87.85377964338281</v>
+        <v>80.28831169169315</v>
       </c>
       <c r="D211" t="n">
         <v>0</v>
@@ -7167,7 +7167,7 @@
         <v>89</v>
       </c>
       <c r="F232" t="n">
-        <v>29.83118998594982</v>
+        <v>32.23595134491106</v>
       </c>
       <c r="G232" t="n">
         <v>1.731</v>
@@ -7956,7 +7956,7 @@
         <v>0.296</v>
       </c>
       <c r="H259" t="n">
-        <v>34.18356335809587</v>
+        <v>37.08398133955755</v>
       </c>
       <c r="I259" t="n">
         <v>1</v>
@@ -8086,7 +8086,7 @@
         <v>116</v>
       </c>
       <c r="C264" t="n">
-        <v>62.98474970449496</v>
+        <v>67.16263458966424</v>
       </c>
       <c r="D264" t="n">
         <v>0</v>
@@ -8202,7 +8202,7 @@
         <v>119</v>
       </c>
       <c r="C268" t="n">
-        <v>66.56709634877241</v>
+        <v>69.62256447280738</v>
       </c>
       <c r="D268" t="n">
         <v>0</v>
@@ -8260,7 +8260,7 @@
         <v>96</v>
       </c>
       <c r="C270" t="n">
-        <v>76.75434607946727</v>
+        <v>69.40540589628912</v>
       </c>
       <c r="D270" t="n">
         <v>0</v>
@@ -8382,7 +8382,7 @@
         <v>14</v>
       </c>
       <c r="E274" t="n">
-        <v>154.7385900032754</v>
+        <v>82.56504050820924</v>
       </c>
       <c r="F274" t="n">
         <v>23.7</v>
@@ -9217,7 +9217,7 @@
         <v>73</v>
       </c>
       <c r="C303" t="n">
-        <v>62.60922067270496</v>
+        <v>64.75679712861688</v>
       </c>
       <c r="D303" t="n">
         <v>0</v>
@@ -9246,7 +9246,7 @@
         <v>90</v>
       </c>
       <c r="C304" t="n">
-        <v>71.92709007745879</v>
+        <v>70.93534193700513</v>
       </c>
       <c r="D304" t="n">
         <v>0</v>
@@ -10000,7 +10000,7 @@
         <v>135</v>
       </c>
       <c r="C330" t="n">
-        <v>85.14548264745889</v>
+        <v>86.13750553077915</v>
       </c>
       <c r="D330" t="n">
         <v>0</v>
@@ -10435,7 +10435,7 @@
         <v>167</v>
       </c>
       <c r="C345" t="n">
-        <v>76.13531722806758</v>
+        <v>72.36952266858566</v>
       </c>
       <c r="D345" t="n">
         <v>0</v>
@@ -10493,7 +10493,7 @@
         <v>117</v>
       </c>
       <c r="C347" t="n">
-        <v>80.01743972501092</v>
+        <v>75.88783205894705</v>
       </c>
       <c r="D347" t="n">
         <v>0</v>
@@ -11363,7 +11363,7 @@
         <v>115</v>
       </c>
       <c r="C377" t="n">
-        <v>77.34293705743073</v>
+        <v>75.90269346429211</v>
       </c>
       <c r="D377" t="n">
         <v>0</v>
@@ -11479,7 +11479,7 @@
         <v>129</v>
       </c>
       <c r="C381" t="n">
-        <v>82.36195690979226</v>
+        <v>77.79029554633877</v>
       </c>
       <c r="D381" t="n">
         <v>0</v>
@@ -12668,7 +12668,7 @@
         <v>146</v>
       </c>
       <c r="C422" t="n">
-        <v>74.80538362899159</v>
+        <v>70.35767205474076</v>
       </c>
       <c r="D422" t="n">
         <v>0</v>
@@ -13103,7 +13103,7 @@
         <v>115</v>
       </c>
       <c r="C437" t="n">
-        <v>76.92959604042187</v>
+        <v>74.05807736893721</v>
       </c>
       <c r="D437" t="n">
         <v>0</v>
@@ -13112,7 +13112,7 @@
         <v>0</v>
       </c>
       <c r="F437" t="n">
-        <v>31.21969709833307</v>
+        <v>29.47418928418386</v>
       </c>
       <c r="G437" t="n">
         <v>0.261</v>
@@ -13161,7 +13161,7 @@
         <v>87</v>
       </c>
       <c r="C439" t="n">
-        <v>63.07945518241306</v>
+        <v>69.53179254135648</v>
       </c>
       <c r="D439" t="n">
         <v>23</v>
@@ -13738,7 +13738,7 @@
         <v>5</v>
       </c>
       <c r="B459" t="n">
-        <v>116.1983393381533</v>
+        <v>120.3226808994161</v>
       </c>
       <c r="C459" t="n">
         <v>80</v>
@@ -13982,7 +13982,7 @@
         <v>20</v>
       </c>
       <c r="E6" t="n">
-        <v>3.537281908660711</v>
+        <v>3.640338244091948</v>
       </c>
       <c r="F6" t="n">
         <v>24.4</v>
@@ -15281,7 +15281,7 @@
         <v>183</v>
       </c>
       <c r="C51" t="n">
-        <v>4.358260764369001</v>
+        <v>4.325519161341184</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
@@ -15539,7 +15539,7 @@
         <v>1</v>
       </c>
       <c r="B60" t="n">
-        <v>90.62035702479233</v>
+        <v>104.7970651670725</v>
       </c>
       <c r="C60" t="n">
         <v>4.31748811353631</v>
@@ -15571,7 +15571,7 @@
         <v>146</v>
       </c>
       <c r="C61" t="n">
-        <v>4.354906016715073</v>
+        <v>4.284561594896813</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
@@ -15580,7 +15580,7 @@
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>31.72671117694619</v>
+        <v>30.81547598881929</v>
       </c>
       <c r="G61" t="n">
         <v>0.4898979485566356</v>
@@ -16586,7 +16586,7 @@
         <v>129</v>
       </c>
       <c r="C96" t="n">
-        <v>4.720902488289525</v>
+        <v>4.448755339045245</v>
       </c>
       <c r="D96" t="n">
         <v>30</v>
@@ -17166,7 +17166,7 @@
         <v>120</v>
       </c>
       <c r="C116" t="n">
-        <v>4.345905944686333</v>
+        <v>4.342802731697334</v>
       </c>
       <c r="D116" t="n">
         <v>0</v>
@@ -18384,7 +18384,7 @@
         <v>114</v>
       </c>
       <c r="C158" t="n">
-        <v>4.26882729871391</v>
+        <v>4.280457284161717</v>
       </c>
       <c r="D158" t="n">
         <v>0</v>
@@ -18393,7 +18393,7 @@
         <v>0</v>
       </c>
       <c r="F158" t="n">
-        <v>29.90296691495914</v>
+        <v>29.31107299630873</v>
       </c>
       <c r="G158" t="n">
         <v>0.4347413023856831</v>
@@ -18587,7 +18587,7 @@
         <v>141</v>
       </c>
       <c r="C165" t="n">
-        <v>4.314041454884618</v>
+        <v>4.279970088497767</v>
       </c>
       <c r="D165" t="n">
         <v>0</v>
@@ -18964,7 +18964,7 @@
         <v>80</v>
       </c>
       <c r="C178" t="n">
-        <v>4.211452158370609</v>
+        <v>4.227610383476766</v>
       </c>
       <c r="D178" t="n">
         <v>0</v>
@@ -18973,7 +18973,7 @@
         <v>0</v>
       </c>
       <c r="F178" t="n">
-        <v>29.35369501897569</v>
+        <v>27.5349765300166</v>
       </c>
       <c r="G178" t="n">
         <v>0.4171330722922842</v>
@@ -19341,7 +19341,7 @@
         <v>100</v>
       </c>
       <c r="C191" t="n">
-        <v>4.272586237925015</v>
+        <v>4.308632037611828</v>
       </c>
       <c r="D191" t="n">
         <v>0</v>
@@ -19570,7 +19570,7 @@
         <v>1</v>
       </c>
       <c r="B199" t="n">
-        <v>104.4851832149699</v>
+        <v>101.9041563643626</v>
       </c>
       <c r="C199" t="n">
         <v>4.23410650459726</v>
@@ -19921,7 +19921,7 @@
         <v>180</v>
       </c>
       <c r="C211" t="n">
-        <v>4.486992093295008</v>
+        <v>4.398002238588358</v>
       </c>
       <c r="D211" t="n">
         <v>0</v>
@@ -20539,7 +20539,7 @@
         <v>4.499809670330265</v>
       </c>
       <c r="F232" t="n">
-        <v>29.83118998594982</v>
+        <v>32.23595134491106</v>
       </c>
       <c r="G232" t="n">
         <v>1.315674731839143</v>
@@ -21328,7 +21328,7 @@
         <v>0.5440588203494178</v>
       </c>
       <c r="H259" t="n">
-        <v>5.846671134765138</v>
+        <v>6.08966184114993</v>
       </c>
       <c r="I259" t="n">
         <v>1</v>
@@ -21458,7 +21458,7 @@
         <v>116</v>
       </c>
       <c r="C264" t="n">
-        <v>4.158644769097817</v>
+        <v>4.221896534791426</v>
       </c>
       <c r="D264" t="n">
         <v>0</v>
@@ -21574,7 +21574,7 @@
         <v>119</v>
       </c>
       <c r="C268" t="n">
-        <v>4.213121124149581</v>
+        <v>4.257349703531191</v>
       </c>
       <c r="D268" t="n">
         <v>0</v>
@@ -21632,7 +21632,7 @@
         <v>96</v>
       </c>
       <c r="C270" t="n">
-        <v>4.353554447625298</v>
+        <v>4.254270048515488</v>
       </c>
       <c r="D270" t="n">
         <v>0</v>
@@ -21754,7 +21754,7 @@
         <v>14</v>
       </c>
       <c r="E274" t="n">
-        <v>5.048178896578098</v>
+        <v>4.425625256891674</v>
       </c>
       <c r="F274" t="n">
         <v>23.7</v>
@@ -22589,7 +22589,7 @@
         <v>73</v>
       </c>
       <c r="C303" t="n">
-        <v>4.152758438968199</v>
+        <v>4.185963044096703</v>
       </c>
       <c r="D303" t="n">
         <v>0</v>
@@ -22618,7 +22618,7 @@
         <v>90</v>
       </c>
       <c r="C304" t="n">
-        <v>4.289460175987009</v>
+        <v>4.275767686894049</v>
       </c>
       <c r="D304" t="n">
         <v>0</v>
@@ -23372,7 +23372,7 @@
         <v>135</v>
       </c>
       <c r="C330" t="n">
-        <v>4.45603752570196</v>
+        <v>4.467487394284374</v>
       </c>
       <c r="D330" t="n">
         <v>0</v>
@@ -23807,7 +23807,7 @@
         <v>167</v>
       </c>
       <c r="C345" t="n">
-        <v>4.345561246090016</v>
+        <v>4.295508626892905</v>
       </c>
       <c r="D345" t="n">
         <v>0</v>
@@ -23865,7 +23865,7 @@
         <v>117</v>
       </c>
       <c r="C347" t="n">
-        <v>4.394664436744638</v>
+        <v>4.342347633288901</v>
       </c>
       <c r="D347" t="n">
         <v>0</v>
@@ -24735,7 +24735,7 @@
         <v>115</v>
       </c>
       <c r="C377" t="n">
-        <v>4.361095818694352</v>
+        <v>4.342540901441679</v>
       </c>
       <c r="D377" t="n">
         <v>0</v>
@@ -24851,7 +24851,7 @@
         <v>129</v>
       </c>
       <c r="C381" t="n">
-        <v>4.423192053134891</v>
+        <v>4.36678983631464</v>
       </c>
       <c r="D381" t="n">
         <v>0</v>
@@ -26040,7 +26040,7 @@
         <v>146</v>
       </c>
       <c r="C422" t="n">
-        <v>4.328169314255408</v>
+        <v>4.267704865188349</v>
       </c>
       <c r="D422" t="n">
         <v>0</v>
@@ -26475,7 +26475,7 @@
         <v>115</v>
       </c>
       <c r="C437" t="n">
-        <v>4.355805804221117</v>
+        <v>4.31826217878965</v>
       </c>
       <c r="D437" t="n">
         <v>0</v>
@@ -26484,7 +26484,7 @@
         <v>0</v>
       </c>
       <c r="F437" t="n">
-        <v>31.21969709833307</v>
+        <v>29.47418928418386</v>
       </c>
       <c r="G437" t="n">
         <v>0.5108815909777921</v>
@@ -26533,7 +26533,7 @@
         <v>87</v>
       </c>
       <c r="C439" t="n">
-        <v>4.160123800576848</v>
+        <v>4.256063566200633</v>
       </c>
       <c r="D439" t="n">
         <v>23</v>
@@ -27110,7 +27110,7 @@
         <v>5</v>
       </c>
       <c r="B459" t="n">
-        <v>116.1983393381533</v>
+        <v>120.3226808994161</v>
       </c>
       <c r="C459" t="n">
         <v>4.394449154672439</v>
@@ -27722,7 +27722,7 @@
         <v>6</v>
       </c>
       <c r="B19" t="n">
-        <v>113.7690510827053</v>
+        <v>118.0566195734959</v>
       </c>
       <c r="C19" t="n">
         <v>68</v>
@@ -28740,7 +28740,7 @@
         <v>105</v>
       </c>
       <c r="C54" t="n">
-        <v>66.47726974050731</v>
+        <v>70.71505801387372</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
@@ -28749,7 +28749,7 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>30.17796755797328</v>
+        <v>28.87787923790112</v>
       </c>
       <c r="G54" t="n">
         <v>0.305</v>
@@ -29001,7 +29001,7 @@
         <v>91</v>
       </c>
       <c r="C63" t="n">
-        <v>70.52123229836869</v>
+        <v>72.38992198713792</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
@@ -29175,7 +29175,7 @@
         <v>132</v>
       </c>
       <c r="C69" t="n">
-        <v>71.3328529693633</v>
+        <v>71.33641743924096</v>
       </c>
       <c r="D69" t="n">
         <v>0</v>
@@ -29204,7 +29204,7 @@
         <v>119</v>
       </c>
       <c r="C70" t="n">
-        <v>70.02872435783222</v>
+        <v>79.66366622070426</v>
       </c>
       <c r="D70" t="n">
         <v>0</v>
@@ -29764,7 +29764,7 @@
         <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>31.67332210896627</v>
+        <v>30.65265279472035</v>
       </c>
       <c r="G89" t="n">
         <v>0.232</v>
@@ -29909,7 +29909,7 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
-        <v>33.01334405579803</v>
+        <v>30.50890022167927</v>
       </c>
       <c r="G94" t="n">
         <v>0.64</v>
@@ -30219,13 +30219,13 @@
         <v>99</v>
       </c>
       <c r="C105" t="n">
-        <v>62.09241930618673</v>
+        <v>65.83592458203489</v>
       </c>
       <c r="D105" t="n">
         <v>0</v>
       </c>
       <c r="E105" t="n">
-        <v>0.02898989898989899</v>
+        <v>6.981496160481868</v>
       </c>
       <c r="F105" t="n">
         <v>22.2</v>
@@ -31118,7 +31118,7 @@
         <v>84</v>
       </c>
       <c r="C136" t="n">
-        <v>66.7845500006606</v>
+        <v>67.02312693239526</v>
       </c>
       <c r="D136" t="n">
         <v>0</v>
@@ -31127,7 +31127,7 @@
         <v>0</v>
       </c>
       <c r="F136" t="n">
-        <v>30.17731149357194</v>
+        <v>27.70521073365259</v>
       </c>
       <c r="G136" t="n">
         <v>0.304</v>
@@ -31408,7 +31408,7 @@
         <v>119</v>
       </c>
       <c r="C146" t="n">
-        <v>71.34521906896266</v>
+        <v>73.46735148851246</v>
       </c>
       <c r="D146" t="n">
         <v>0</v>
@@ -31466,7 +31466,7 @@
         <v>94</v>
       </c>
       <c r="C148" t="n">
-        <v>66.39636368531437</v>
+        <v>67.81209931132021</v>
       </c>
       <c r="D148" t="n">
         <v>0</v>
@@ -31475,7 +31475,7 @@
         <v>0</v>
       </c>
       <c r="F148" t="n">
-        <v>28.43844896931094</v>
+        <v>28.17527754494255</v>
       </c>
       <c r="G148" t="n">
         <v>0.256</v>
@@ -31495,7 +31495,7 @@
         <v>141</v>
       </c>
       <c r="C149" t="n">
-        <v>80.31627992612464</v>
+        <v>75.22094797627892</v>
       </c>
       <c r="D149" t="n">
         <v>0</v>
@@ -32220,7 +32220,7 @@
         <v>6</v>
       </c>
       <c r="B19" t="n">
-        <v>113.7690510827053</v>
+        <v>118.0566195734959</v>
       </c>
       <c r="C19" t="n">
         <v>68</v>
@@ -33238,7 +33238,7 @@
         <v>105</v>
       </c>
       <c r="C54" t="n">
-        <v>66.47726974050731</v>
+        <v>70.71505801387372</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
@@ -33247,7 +33247,7 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>30.17796755797328</v>
+        <v>28.87787923790112</v>
       </c>
       <c r="G54" t="n">
         <v>0.305</v>
@@ -33499,7 +33499,7 @@
         <v>91</v>
       </c>
       <c r="C63" t="n">
-        <v>70.52123229836869</v>
+        <v>72.38992198713792</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
@@ -33673,7 +33673,7 @@
         <v>132</v>
       </c>
       <c r="C69" t="n">
-        <v>71.3328529693633</v>
+        <v>71.33641743924096</v>
       </c>
       <c r="D69" t="n">
         <v>0</v>
@@ -33702,7 +33702,7 @@
         <v>119</v>
       </c>
       <c r="C70" t="n">
-        <v>70.02872435783222</v>
+        <v>79.66366622070426</v>
       </c>
       <c r="D70" t="n">
         <v>0</v>
@@ -34262,7 +34262,7 @@
         <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>31.67332210896627</v>
+        <v>30.65265279472035</v>
       </c>
       <c r="G89" t="n">
         <v>0.232</v>
@@ -34407,7 +34407,7 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
-        <v>33.01334405579803</v>
+        <v>30.50890022167927</v>
       </c>
       <c r="G94" t="n">
         <v>0.64</v>
@@ -34717,13 +34717,13 @@
         <v>99</v>
       </c>
       <c r="C105" t="n">
-        <v>62.09241930618673</v>
+        <v>65.83592458203489</v>
       </c>
       <c r="D105" t="n">
         <v>0</v>
       </c>
       <c r="E105" t="n">
-        <v>0.02898989898989899</v>
+        <v>6.981496160481868</v>
       </c>
       <c r="F105" t="n">
         <v>22.2</v>
@@ -35616,7 +35616,7 @@
         <v>84</v>
       </c>
       <c r="C136" t="n">
-        <v>66.7845500006606</v>
+        <v>67.02312693239526</v>
       </c>
       <c r="D136" t="n">
         <v>0</v>
@@ -35625,7 +35625,7 @@
         <v>0</v>
       </c>
       <c r="F136" t="n">
-        <v>30.17731149357194</v>
+        <v>27.70521073365259</v>
       </c>
       <c r="G136" t="n">
         <v>0.304</v>
@@ -35906,7 +35906,7 @@
         <v>119</v>
       </c>
       <c r="C146" t="n">
-        <v>71.34521906896266</v>
+        <v>73.46735148851246</v>
       </c>
       <c r="D146" t="n">
         <v>0</v>
@@ -35964,7 +35964,7 @@
         <v>94</v>
       </c>
       <c r="C148" t="n">
-        <v>66.39636368531437</v>
+        <v>67.81209931132021</v>
       </c>
       <c r="D148" t="n">
         <v>0</v>
@@ -35973,7 +35973,7 @@
         <v>0</v>
       </c>
       <c r="F148" t="n">
-        <v>28.43844896931094</v>
+        <v>28.17527754494255</v>
       </c>
       <c r="G148" t="n">
         <v>0.256</v>
@@ -35993,7 +35993,7 @@
         <v>141</v>
       </c>
       <c r="C149" t="n">
-        <v>80.31627992612464</v>
+        <v>75.22094797627892</v>
       </c>
       <c r="D149" t="n">
         <v>0</v>
@@ -36286,7 +36286,7 @@
         <v>99</v>
       </c>
       <c r="C4" t="n">
-        <v>63.93935233812172</v>
+        <v>65.88726625802548</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -36344,7 +36344,7 @@
         <v>74</v>
       </c>
       <c r="C6" t="n">
-        <v>64.95349685578375</v>
+        <v>66.92065883845605</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -36353,7 +36353,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>28.06668079543562</v>
+        <v>27.21415684773827</v>
       </c>
       <c r="G6" t="n">
         <v>0.102</v>
@@ -36866,7 +36866,7 @@
         <v>138</v>
       </c>
       <c r="C24" t="n">
-        <v>69.41062780756877</v>
+        <v>71.73348872596816</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -36982,7 +36982,7 @@
         <v>145</v>
       </c>
       <c r="C28" t="n">
-        <v>80.72674791568281</v>
+        <v>76.53589151374399</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -38548,7 +38548,7 @@
         <v>99</v>
       </c>
       <c r="C82" t="n">
-        <v>62.09241930618673</v>
+        <v>65.92914746659666</v>
       </c>
       <c r="D82" t="n">
         <v>0</v>
@@ -39427,7 +39427,7 @@
         <v>0</v>
       </c>
       <c r="F112" t="n">
-        <v>27.94252680312734</v>
+        <v>31.82464887183267</v>
       </c>
       <c r="G112" t="n">
         <v>0.572</v>
@@ -39444,7 +39444,7 @@
         <v>1</v>
       </c>
       <c r="B113" t="n">
-        <v>124.8406270345927</v>
+        <v>112.8724305703829</v>
       </c>
       <c r="C113" t="n">
         <v>98</v>
@@ -39882,7 +39882,7 @@
         <v>131</v>
       </c>
       <c r="C128" t="n">
-        <v>78.3604474321105</v>
+        <v>74.41704384508148</v>
       </c>
       <c r="D128" t="n">
         <v>0</v>
@@ -40372,7 +40372,7 @@
         <v>1</v>
       </c>
       <c r="B145" t="n">
-        <v>103.8879464737581</v>
+        <v>100.0292946013914</v>
       </c>
       <c r="C145" t="n">
         <v>48</v>
@@ -40813,7 +40813,7 @@
         <v>99</v>
       </c>
       <c r="C4" t="n">
-        <v>63.93935233812172</v>
+        <v>65.88726625802548</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -40871,7 +40871,7 @@
         <v>74</v>
       </c>
       <c r="C6" t="n">
-        <v>64.95349685578375</v>
+        <v>66.92065883845605</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -40880,7 +40880,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>28.06668079543562</v>
+        <v>27.21415684773827</v>
       </c>
       <c r="G6" t="n">
         <v>0.102</v>
@@ -41393,7 +41393,7 @@
         <v>138</v>
       </c>
       <c r="C24" t="n">
-        <v>69.41062780756877</v>
+        <v>71.73348872596816</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -41509,7 +41509,7 @@
         <v>145</v>
       </c>
       <c r="C28" t="n">
-        <v>80.72674791568281</v>
+        <v>76.53589151374399</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -43075,7 +43075,7 @@
         <v>99</v>
       </c>
       <c r="C82" t="n">
-        <v>62.09241930618673</v>
+        <v>65.92914746659666</v>
       </c>
       <c r="D82" t="n">
         <v>0</v>
@@ -43954,7 +43954,7 @@
         <v>0</v>
       </c>
       <c r="F112" t="n">
-        <v>27.94252680312734</v>
+        <v>31.82464887183267</v>
       </c>
       <c r="G112" t="n">
         <v>0.572</v>
@@ -43971,7 +43971,7 @@
         <v>1</v>
       </c>
       <c r="B113" t="n">
-        <v>124.8406270345927</v>
+        <v>112.8724305703829</v>
       </c>
       <c r="C113" t="n">
         <v>98</v>
@@ -44409,7 +44409,7 @@
         <v>131</v>
       </c>
       <c r="C128" t="n">
-        <v>78.3604474321105</v>
+        <v>74.41704384508148</v>
       </c>
       <c r="D128" t="n">
         <v>0</v>
@@ -44899,7 +44899,7 @@
         <v>1</v>
       </c>
       <c r="B145" t="n">
-        <v>103.8879464737581</v>
+        <v>100.0292946013914</v>
       </c>
       <c r="C145" t="n">
         <v>48</v>

</xml_diff>